<commit_message>
Atualiza relatórios e gráficos do iGovTI 2026
</commit_message>
<xml_diff>
--- a/02-Execucao/01-Questionario/04-Resultados_iGovTI/03-pos-comentarios-gestor/20260716-iGovTI-2026.xlsx
+++ b/02-Execucao/01-Questionario/04-Resultados_iGovTI/03-pos-comentarios-gestor/20260716-iGovTI-2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M114"/>
+  <dimension ref="A1:Q114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,6 +482,26 @@
           <t>iGestTI</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>q1001</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>q1002</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>q1003</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>q1004</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -527,6 +547,18 @@
       <c r="M2" t="n">
         <v>0.03697048457509202</v>
       </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -572,6 +604,18 @@
       <c r="M3" t="n">
         <v>0.0375236230727873</v>
       </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -617,6 +661,18 @@
       <c r="M4" t="n">
         <v>0.07072715617144382</v>
       </c>
+      <c r="N4" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -662,6 +718,18 @@
       <c r="M5" t="n">
         <v>0.2925989546900496</v>
       </c>
+      <c r="N5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -707,6 +775,18 @@
       <c r="M6" t="n">
         <v>0.1648497088626512</v>
       </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -752,6 +832,18 @@
       <c r="M7" t="n">
         <v>0.3504128688766328</v>
       </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -797,6 +889,18 @@
       <c r="M8" t="n">
         <v>0.1244983321450206</v>
       </c>
+      <c r="N8" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -842,6 +946,18 @@
       <c r="M9" t="n">
         <v>0.3826129239536639</v>
       </c>
+      <c r="N9" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.5142857142857142</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -887,6 +1003,18 @@
       <c r="M10" t="n">
         <v>0.1445358184493309</v>
       </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -932,6 +1060,18 @@
       <c r="M11" t="n">
         <v>0.1411920198943285</v>
       </c>
+      <c r="N11" t="n">
+        <v>0.5277777777777778</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -977,6 +1117,18 @@
       <c r="M12" t="n">
         <v>0.2706315213035547</v>
       </c>
+      <c r="N12" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1022,6 +1174,18 @@
       <c r="M13" t="n">
         <v>0.1428471485440407</v>
       </c>
+      <c r="N13" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1067,6 +1231,18 @@
       <c r="M14" t="n">
         <v>0.4420225287380281</v>
       </c>
+      <c r="N14" t="n">
+        <v>0.7166666666666667</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P14" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0.2000000000000001</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1112,6 +1288,18 @@
       <c r="M15" t="n">
         <v>0.0738066985195609</v>
       </c>
+      <c r="N15" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1157,6 +1345,18 @@
       <c r="M16" t="n">
         <v>0.01900693927304798</v>
       </c>
+      <c r="N16" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1202,6 +1402,18 @@
       <c r="M17" t="n">
         <v>0.04942955913713883</v>
       </c>
+      <c r="N17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1247,6 +1459,18 @@
       <c r="M18" t="n">
         <v>0.1636859938296688</v>
       </c>
+      <c r="N18" t="n">
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1292,6 +1516,18 @@
       <c r="M19" t="n">
         <v>0.1856042163974627</v>
       </c>
+      <c r="N19" t="n">
+        <v>0.3055555555555556</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1337,6 +1573,18 @@
       <c r="M20" t="n">
         <v>0.1507064229561005</v>
       </c>
+      <c r="N20" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1382,6 +1630,18 @@
       <c r="M21" t="n">
         <v>0.2430064122609939</v>
       </c>
+      <c r="N21" t="n">
+        <v>0.2277777777777778</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P21" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1427,6 +1687,18 @@
       <c r="M22" t="n">
         <v>0.1821005343777428</v>
       </c>
+      <c r="N22" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0.6357142857142857</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1472,6 +1744,18 @@
       <c r="M23" t="n">
         <v>0.1852538316721145</v>
       </c>
+      <c r="N23" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1517,6 +1801,18 @@
       <c r="M24" t="n">
         <v>0.09448344060072406</v>
       </c>
+      <c r="N24" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1562,6 +1858,18 @@
       <c r="M25" t="n">
         <v>0.2227310974276348</v>
       </c>
+      <c r="N25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1607,6 +1915,18 @@
       <c r="M26" t="n">
         <v>0.4576038883747021</v>
       </c>
+      <c r="N26" t="n">
+        <v>0.7166666666666667</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0.2375</v>
+      </c>
+      <c r="P26" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>0.2714285714285715</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1652,6 +1972,18 @@
       <c r="M27" t="n">
         <v>0.02795160228020204</v>
       </c>
+      <c r="N27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1697,6 +2029,18 @@
       <c r="M28" t="n">
         <v>0.2800301049159163</v>
       </c>
+      <c r="N28" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1742,6 +2086,18 @@
       <c r="M29" t="n">
         <v>0.09746267550538897</v>
       </c>
+      <c r="N29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1787,6 +2143,18 @@
       <c r="M30" t="n">
         <v>0.3047477962812494</v>
       </c>
+      <c r="N30" t="n">
+        <v>0.3444444444444444</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1832,6 +2200,18 @@
       <c r="M31" t="n">
         <v>0.2931824282310064</v>
       </c>
+      <c r="N31" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1877,6 +2257,18 @@
       <c r="M32" t="n">
         <v>0.008556612942918993</v>
       </c>
+      <c r="N32" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1922,6 +2314,18 @@
       <c r="M33" t="n">
         <v>0</v>
       </c>
+      <c r="N33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1967,6 +2371,18 @@
       <c r="M34" t="n">
         <v>0.04792394356932806</v>
       </c>
+      <c r="N34" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2012,6 +2428,18 @@
       <c r="M35" t="n">
         <v>0.005264756332862353</v>
       </c>
+      <c r="N35" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2057,6 +2485,18 @@
       <c r="M36" t="n">
         <v>0.630685367974276</v>
       </c>
+      <c r="N36" t="n">
+        <v>0.8111111111111111</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0.7875</v>
+      </c>
+      <c r="P36" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2102,6 +2542,18 @@
       <c r="M37" t="n">
         <v>0.09323532853342023</v>
       </c>
+      <c r="N37" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2147,6 +2599,18 @@
       <c r="M38" t="n">
         <v>0.04858003993748611</v>
       </c>
+      <c r="N38" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" t="n">
+        <v>0</v>
+      </c>
+      <c r="P38" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2192,6 +2656,18 @@
       <c r="M39" t="n">
         <v>0.01932468878515482</v>
       </c>
+      <c r="N39" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2237,6 +2713,18 @@
       <c r="M40" t="n">
         <v>0.3080145500533631</v>
       </c>
+      <c r="N40" t="n">
+        <v>0.1888888888888889</v>
+      </c>
+      <c r="O40" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>0.25</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2282,6 +2770,18 @@
       <c r="M41" t="n">
         <v>0.1778895593202559</v>
       </c>
+      <c r="N41" t="n">
+        <v>0.7166666666666667</v>
+      </c>
+      <c r="O41" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>0.2000000000000001</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2327,6 +2827,18 @@
       <c r="M42" t="n">
         <v>0.6916799832697542</v>
       </c>
+      <c r="N42" t="n">
+        <v>0.7166666666666667</v>
+      </c>
+      <c r="O42" t="n">
+        <v>1</v>
+      </c>
+      <c r="P42" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>0.7571428571428571</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2372,6 +2884,18 @@
       <c r="M43" t="n">
         <v>0.6595603441947895</v>
       </c>
+      <c r="N43" t="n">
+        <v>0.9055555555555556</v>
+      </c>
+      <c r="O43" t="n">
+        <v>1</v>
+      </c>
+      <c r="P43" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2417,6 +2941,18 @@
       <c r="M44" t="n">
         <v>0.1935977235291988</v>
       </c>
+      <c r="N44" t="n">
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2462,6 +2998,18 @@
       <c r="M45" t="n">
         <v>0.1197665744431394</v>
       </c>
+      <c r="N45" t="n">
+        <v>0.2277777777777778</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0.2375</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2507,6 +3055,18 @@
       <c r="M46" t="n">
         <v>0.2501537827349325</v>
       </c>
+      <c r="N46" t="n">
+        <v>0.2277777777777778</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>0.2000000000000001</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2552,6 +3112,18 @@
       <c r="M47" t="n">
         <v>0.1192925460334332</v>
       </c>
+      <c r="N47" t="n">
+        <v>0.2277777777777778</v>
+      </c>
+      <c r="O47" t="n">
+        <v>0</v>
+      </c>
+      <c r="P47" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>0.6357142857142857</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2597,6 +3169,18 @@
       <c r="M48" t="n">
         <v>0.1347928255537475</v>
       </c>
+      <c r="N48" t="n">
+        <v>0</v>
+      </c>
+      <c r="O48" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="P48" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2642,6 +3226,18 @@
       <c r="M49" t="n">
         <v>0.1169304395588576</v>
       </c>
+      <c r="N49" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O49" t="n">
+        <v>0</v>
+      </c>
+      <c r="P49" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2687,6 +3283,18 @@
       <c r="M50" t="n">
         <v>0.1089340171689637</v>
       </c>
+      <c r="N50" t="n">
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="O50" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="P50" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2732,6 +3340,18 @@
       <c r="M51" t="n">
         <v>0.4067678246081828</v>
       </c>
+      <c r="N51" t="n">
+        <v>1</v>
+      </c>
+      <c r="O51" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2777,6 +3397,18 @@
       <c r="M52" t="n">
         <v>0.1814116983449462</v>
       </c>
+      <c r="N52" t="n">
+        <v>0.1888888888888889</v>
+      </c>
+      <c r="O52" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P52" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2822,6 +3454,18 @@
       <c r="M53" t="n">
         <v>0.1548577497047572</v>
       </c>
+      <c r="N53" t="n">
+        <v>0.2277777777777778</v>
+      </c>
+      <c r="O53" t="n">
+        <v>0</v>
+      </c>
+      <c r="P53" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2867,6 +3511,18 @@
       <c r="M54" t="n">
         <v>0</v>
       </c>
+      <c r="N54" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" t="n">
+        <v>0</v>
+      </c>
+      <c r="P54" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2912,6 +3568,18 @@
       <c r="M55" t="n">
         <v>0.4034893895862416</v>
       </c>
+      <c r="N55" t="n">
+        <v>0.3444444444444444</v>
+      </c>
+      <c r="O55" t="n">
+        <v>0.4125</v>
+      </c>
+      <c r="P55" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2957,6 +3625,18 @@
       <c r="M56" t="n">
         <v>0.182647852810813</v>
       </c>
+      <c r="N56" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P56" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3002,6 +3682,18 @@
       <c r="M57" t="n">
         <v>0.2672739598415609</v>
       </c>
+      <c r="N57" t="n">
+        <v>0.4333333333333333</v>
+      </c>
+      <c r="O57" t="n">
+        <v>0</v>
+      </c>
+      <c r="P57" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3047,6 +3739,18 @@
       <c r="M58" t="n">
         <v>0.1171904423089602</v>
       </c>
+      <c r="N58" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O58" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P58" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3092,6 +3796,18 @@
       <c r="M59" t="n">
         <v>0.1825218531967478</v>
       </c>
+      <c r="N59" t="n">
+        <v>0.6222222222222222</v>
+      </c>
+      <c r="O59" t="n">
+        <v>0</v>
+      </c>
+      <c r="P59" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>0.5142857142857142</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3137,6 +3853,18 @@
       <c r="M60" t="n">
         <v>0.04942955913713883</v>
       </c>
+      <c r="N60" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O60" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="P60" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3182,6 +3910,18 @@
       <c r="M61" t="n">
         <v>0.1026364961242728</v>
       </c>
+      <c r="N61" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O61" t="n">
+        <v>0</v>
+      </c>
+      <c r="P61" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3227,6 +3967,18 @@
       <c r="M62" t="n">
         <v>0.1123135487254382</v>
       </c>
+      <c r="N62" t="n">
+        <v>0</v>
+      </c>
+      <c r="O62" t="n">
+        <v>0</v>
+      </c>
+      <c r="P62" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3272,6 +4024,18 @@
       <c r="M63" t="n">
         <v>0.1048394425216523</v>
       </c>
+      <c r="N63" t="n">
+        <v>0</v>
+      </c>
+      <c r="O63" t="n">
+        <v>0</v>
+      </c>
+      <c r="P63" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3317,6 +4081,18 @@
       <c r="M64" t="n">
         <v>0.104812080348367</v>
       </c>
+      <c r="N64" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O64" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P64" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3362,6 +4138,18 @@
       <c r="M65" t="n">
         <v>0.0948223192781862</v>
       </c>
+      <c r="N65" t="n">
+        <v>0.2444444444444445</v>
+      </c>
+      <c r="O65" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="P65" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3407,6 +4195,18 @@
       <c r="M66" t="n">
         <v>0.05795802129230847</v>
       </c>
+      <c r="N66" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O66" t="n">
+        <v>0</v>
+      </c>
+      <c r="P66" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3452,6 +4252,18 @@
       <c r="M67" t="n">
         <v>0.6964039318488351</v>
       </c>
+      <c r="N67" t="n">
+        <v>0</v>
+      </c>
+      <c r="O67" t="n">
+        <v>1</v>
+      </c>
+      <c r="P67" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>0.2714285714285715</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3497,6 +4309,18 @@
       <c r="M68" t="n">
         <v>0.0905371647110242</v>
       </c>
+      <c r="N68" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O68" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P68" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3542,6 +4366,18 @@
       <c r="M69" t="n">
         <v>0.8016241195599404</v>
       </c>
+      <c r="N69" t="n">
+        <v>1</v>
+      </c>
+      <c r="O69" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P69" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>0.6357142857142857</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3587,6 +4423,18 @@
       <c r="M70" t="n">
         <v>0.1916120538423874</v>
       </c>
+      <c r="N70" t="n">
+        <v>0.2277777777777778</v>
+      </c>
+      <c r="O70" t="n">
+        <v>0</v>
+      </c>
+      <c r="P70" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3632,6 +4480,18 @@
       <c r="M71" t="n">
         <v>0.4660710671287835</v>
       </c>
+      <c r="N71" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O71" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P71" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3677,6 +4537,18 @@
       <c r="M72" t="n">
         <v>0.08215176001564206</v>
       </c>
+      <c r="N72" t="n">
+        <v>0</v>
+      </c>
+      <c r="O72" t="n">
+        <v>0</v>
+      </c>
+      <c r="P72" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3722,6 +4594,18 @@
       <c r="M73" t="n">
         <v>0.3358962417910585</v>
       </c>
+      <c r="N73" t="n">
+        <v>0</v>
+      </c>
+      <c r="O73" t="n">
+        <v>0</v>
+      </c>
+      <c r="P73" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>0.35</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3767,6 +4651,18 @@
       <c r="M74" t="n">
         <v>0.136811280671431</v>
       </c>
+      <c r="N74" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O74" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P74" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3812,6 +4708,18 @@
       <c r="M75" t="n">
         <v>0</v>
       </c>
+      <c r="N75" t="n">
+        <v>0</v>
+      </c>
+      <c r="O75" t="n">
+        <v>0</v>
+      </c>
+      <c r="P75" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3857,6 +4765,18 @@
       <c r="M76" t="n">
         <v>0</v>
       </c>
+      <c r="N76" t="n">
+        <v>0</v>
+      </c>
+      <c r="O76" t="n">
+        <v>0</v>
+      </c>
+      <c r="P76" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>0.35</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3902,6 +4822,18 @@
       <c r="M77" t="n">
         <v>0.2195959431644446</v>
       </c>
+      <c r="N77" t="n">
+        <v>0.4333333333333333</v>
+      </c>
+      <c r="O77" t="n">
+        <v>0</v>
+      </c>
+      <c r="P77" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3947,6 +4879,18 @@
       <c r="M78" t="n">
         <v>0.7956931926285407</v>
       </c>
+      <c r="N78" t="n">
+        <v>0.8111111111111111</v>
+      </c>
+      <c r="O78" t="n">
+        <v>0.7875</v>
+      </c>
+      <c r="P78" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3992,6 +4936,18 @@
       <c r="M79" t="n">
         <v>0.4257888327452301</v>
       </c>
+      <c r="N79" t="n">
+        <v>0.3444444444444444</v>
+      </c>
+      <c r="O79" t="n">
+        <v>0</v>
+      </c>
+      <c r="P79" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4037,6 +4993,18 @@
       <c r="M80" t="n">
         <v>0.1329752470285211</v>
       </c>
+      <c r="N80" t="n">
+        <v>0.3055555555555556</v>
+      </c>
+      <c r="O80" t="n">
+        <v>0</v>
+      </c>
+      <c r="P80" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4082,6 +5050,18 @@
       <c r="M81" t="n">
         <v>0</v>
       </c>
+      <c r="N81" t="n">
+        <v>0</v>
+      </c>
+      <c r="O81" t="n">
+        <v>0</v>
+      </c>
+      <c r="P81" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4127,6 +5107,18 @@
       <c r="M82" t="n">
         <v>0.2846445866501157</v>
       </c>
+      <c r="N82" t="n">
+        <v>0</v>
+      </c>
+      <c r="O82" t="n">
+        <v>0</v>
+      </c>
+      <c r="P82" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4172,6 +5164,18 @@
       <c r="M83" t="n">
         <v>0</v>
       </c>
+      <c r="N83" t="n">
+        <v>0</v>
+      </c>
+      <c r="O83" t="n">
+        <v>0</v>
+      </c>
+      <c r="P83" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q83" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4217,6 +5221,18 @@
       <c r="M84" t="n">
         <v>0.197782331568332</v>
       </c>
+      <c r="N84" t="n">
+        <v>0.4333333333333333</v>
+      </c>
+      <c r="O84" t="n">
+        <v>0</v>
+      </c>
+      <c r="P84" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q84" t="n">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4262,6 +5278,18 @@
       <c r="M85" t="n">
         <v>0.124841776946916</v>
       </c>
+      <c r="N85" t="n">
+        <v>0</v>
+      </c>
+      <c r="O85" t="n">
+        <v>0</v>
+      </c>
+      <c r="P85" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q85" t="n">
+        <v>0.2000000000000001</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4307,6 +5335,18 @@
       <c r="M86" t="n">
         <v>0.3343606802148462</v>
       </c>
+      <c r="N86" t="n">
+        <v>0.8111111111111111</v>
+      </c>
+      <c r="O86" t="n">
+        <v>0</v>
+      </c>
+      <c r="P86" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="Q86" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4352,6 +5392,18 @@
       <c r="M87" t="n">
         <v>0.07869427490233423</v>
       </c>
+      <c r="N87" t="n">
+        <v>0.2277777777777778</v>
+      </c>
+      <c r="O87" t="n">
+        <v>0</v>
+      </c>
+      <c r="P87" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q87" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4397,6 +5449,18 @@
       <c r="M88" t="n">
         <v>0.2965349121203979</v>
       </c>
+      <c r="N88" t="n">
+        <v>0.6222222222222222</v>
+      </c>
+      <c r="O88" t="n">
+        <v>0</v>
+      </c>
+      <c r="P88" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="Q88" t="n">
+        <v>0.8785714285714286</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4442,6 +5506,18 @@
       <c r="M89" t="n">
         <v>0.0253663722657696</v>
       </c>
+      <c r="N89" t="n">
+        <v>0</v>
+      </c>
+      <c r="O89" t="n">
+        <v>0</v>
+      </c>
+      <c r="P89" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4487,6 +5563,18 @@
       <c r="M90" t="n">
         <v>0.1002699075407856</v>
       </c>
+      <c r="N90" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O90" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P90" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q90" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4532,6 +5620,18 @@
       <c r="M91" t="n">
         <v>0.3090082486152058</v>
       </c>
+      <c r="N91" t="n">
+        <v>0.4333333333333333</v>
+      </c>
+      <c r="O91" t="n">
+        <v>0</v>
+      </c>
+      <c r="P91" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Q91" t="n">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4577,6 +5677,18 @@
       <c r="M92" t="n">
         <v>0.4998001563633294</v>
       </c>
+      <c r="N92" t="n">
+        <v>0</v>
+      </c>
+      <c r="O92" t="n">
+        <v>0</v>
+      </c>
+      <c r="P92" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q92" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4622,6 +5734,18 @@
       <c r="M93" t="n">
         <v>0.2257295289243203</v>
       </c>
+      <c r="N93" t="n">
+        <v>0</v>
+      </c>
+      <c r="O93" t="n">
+        <v>0.4125</v>
+      </c>
+      <c r="P93" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q93" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4667,6 +5791,18 @@
       <c r="M94" t="n">
         <v>0.07777277505130466</v>
       </c>
+      <c r="N94" t="n">
+        <v>0</v>
+      </c>
+      <c r="O94" t="n">
+        <v>0</v>
+      </c>
+      <c r="P94" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q94" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4712,6 +5848,18 @@
       <c r="M95" t="n">
         <v>0.08171634449330044</v>
       </c>
+      <c r="N95" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O95" t="n">
+        <v>0</v>
+      </c>
+      <c r="P95" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q95" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4757,6 +5905,18 @@
       <c r="M96" t="n">
         <v>0.1554117255232419</v>
       </c>
+      <c r="N96" t="n">
+        <v>0</v>
+      </c>
+      <c r="O96" t="n">
+        <v>0</v>
+      </c>
+      <c r="P96" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q96" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4802,6 +5962,18 @@
       <c r="M97" t="n">
         <v>0.07108441743967478</v>
       </c>
+      <c r="N97" t="n">
+        <v>0</v>
+      </c>
+      <c r="O97" t="n">
+        <v>0</v>
+      </c>
+      <c r="P97" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4847,6 +6019,18 @@
       <c r="M98" t="n">
         <v>0.6797104199177266</v>
       </c>
+      <c r="N98" t="n">
+        <v>0.9055555555555556</v>
+      </c>
+      <c r="O98" t="n">
+        <v>1</v>
+      </c>
+      <c r="P98" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="Q98" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4892,6 +6076,18 @@
       <c r="M99" t="n">
         <v>0.04533422501750872</v>
       </c>
+      <c r="N99" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O99" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="P99" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q99" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4937,6 +6133,18 @@
       <c r="M100" t="n">
         <v>0.2689155800743886</v>
       </c>
+      <c r="N100" t="n">
+        <v>0.2277777777777778</v>
+      </c>
+      <c r="O100" t="n">
+        <v>1</v>
+      </c>
+      <c r="P100" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4982,6 +6190,18 @@
       <c r="M101" t="n">
         <v>0.2413689886454244</v>
       </c>
+      <c r="N101" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O101" t="n">
+        <v>0</v>
+      </c>
+      <c r="P101" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q101" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -5027,6 +6247,18 @@
       <c r="M102" t="n">
         <v>0.1178452538988563</v>
       </c>
+      <c r="N102" t="n">
+        <v>0</v>
+      </c>
+      <c r="O102" t="n">
+        <v>0</v>
+      </c>
+      <c r="P102" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5072,6 +6304,18 @@
       <c r="M103" t="n">
         <v>0.2449270545990555</v>
       </c>
+      <c r="N103" t="n">
+        <v>0</v>
+      </c>
+      <c r="O103" t="n">
+        <v>0</v>
+      </c>
+      <c r="P103" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="Q103" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -5117,6 +6361,18 @@
       <c r="M104" t="n">
         <v>0.2775646508155453</v>
       </c>
+      <c r="N104" t="n">
+        <v>0</v>
+      </c>
+      <c r="O104" t="n">
+        <v>0</v>
+      </c>
+      <c r="P104" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q104" t="n">
+        <v>0.8785714285714286</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -5162,6 +6418,18 @@
       <c r="M105" t="n">
         <v>0.5037548572007281</v>
       </c>
+      <c r="N105" t="n">
+        <v>0</v>
+      </c>
+      <c r="O105" t="n">
+        <v>0</v>
+      </c>
+      <c r="P105" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q105" t="n">
+        <v>0.7571428571428571</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -5207,6 +6475,18 @@
       <c r="M106" t="n">
         <v>0.1667681678554963</v>
       </c>
+      <c r="N106" t="n">
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="O106" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="P106" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q106" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5252,6 +6532,18 @@
       <c r="M107" t="n">
         <v>0.2666496395137506</v>
       </c>
+      <c r="N107" t="n">
+        <v>0.3444444444444444</v>
+      </c>
+      <c r="O107" t="n">
+        <v>0</v>
+      </c>
+      <c r="P107" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="Q107" t="n">
+        <v>0.25</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -5297,6 +6589,18 @@
       <c r="M108" t="n">
         <v>0.04726944990486049</v>
       </c>
+      <c r="N108" t="n">
+        <v>0</v>
+      </c>
+      <c r="O108" t="n">
+        <v>0</v>
+      </c>
+      <c r="P108" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q108" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -5342,6 +6646,18 @@
       <c r="M109" t="n">
         <v>0.3759729108713883</v>
       </c>
+      <c r="N109" t="n">
+        <v>0.4333333333333333</v>
+      </c>
+      <c r="O109" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P109" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q109" t="n">
+        <v>0.5142857142857142</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -5387,6 +6703,18 @@
       <c r="M110" t="n">
         <v>0.08643160391026779</v>
       </c>
+      <c r="N110" t="n">
+        <v>0</v>
+      </c>
+      <c r="O110" t="n">
+        <v>0</v>
+      </c>
+      <c r="P110" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q110" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -5432,6 +6760,18 @@
       <c r="M111" t="n">
         <v>0.0208701111230444</v>
       </c>
+      <c r="N111" t="n">
+        <v>0</v>
+      </c>
+      <c r="O111" t="n">
+        <v>0</v>
+      </c>
+      <c r="P111" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q111" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -5477,6 +6817,18 @@
       <c r="M112" t="n">
         <v>0.7172638476075258</v>
       </c>
+      <c r="N112" t="n">
+        <v>0.9055555555555556</v>
+      </c>
+      <c r="O112" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="P112" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="Q112" t="n">
+        <v>0.6357142857142857</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -5522,6 +6874,18 @@
       <c r="M113" t="n">
         <v>0.473649785925013</v>
       </c>
+      <c r="N113" t="n">
+        <v>0.7166666666666667</v>
+      </c>
+      <c r="O113" t="n">
+        <v>0.3625</v>
+      </c>
+      <c r="P113" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="Q113" t="n">
+        <v>0.2000000000000001</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -5566,6 +6930,18 @@
       </c>
       <c r="M114" t="n">
         <v>0.07543698221223774</v>
+      </c>
+      <c r="N114" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O114" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P114" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q114" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>